<commit_message>
Update Fee Schedule Automation Tracker.xlsx
</commit_message>
<xml_diff>
--- a/Fee Schedule Automation Tracker.xlsx
+++ b/Fee Schedule Automation Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://petauri-my.sharepoint.com/personal/wonmin_song_petauri_com/Documents/Desktop/Fee-Schedule-Automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{D9BA4A1E-E287-2A46-A929-6B1241EC5EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A55ECFA-8EB2-486A-B411-41DFEB81824F}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{D9BA4A1E-E287-2A46-A929-6B1241EC5EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36539664-FE04-43C9-B0D3-C504589B307F}"/>
   <bookViews>
-    <workbookView xWindow="8950" yWindow="0" windowWidth="16760" windowHeight="13770" xr2:uid="{7FB893FB-0A35-7B43-A2AE-2994BFE54B15}"/>
+    <workbookView xWindow="4040" yWindow="0" windowWidth="15150" windowHeight="11370" xr2:uid="{7FB893FB-0A35-7B43-A2AE-2994BFE54B15}"/>
   </bookViews>
   <sheets>
     <sheet name="Working Tab" sheetId="1" r:id="rId1"/>
@@ -1199,7 +1199,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1306,9 +1306,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1316,6 +1313,15 @@
     </xf>
     <xf numFmtId="9" fontId="9" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1852,7 +1858,7 @@
       <c r="M2" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="N2" s="33" t="s">
+      <c r="N2" s="32" t="s">
         <v>15</v>
       </c>
       <c r="O2" s="24" t="s">
@@ -1891,7 +1897,7 @@
       <c r="M3" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="N3" s="33" t="s">
+      <c r="N3" s="32" t="s">
         <v>20</v>
       </c>
       <c r="O3" s="24" t="s">
@@ -1930,7 +1936,7 @@
       <c r="M4" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="N4" s="33" t="s">
+      <c r="N4" s="32" t="s">
         <v>25</v>
       </c>
       <c r="O4" s="24" t="s">
@@ -1971,7 +1977,7 @@
       <c r="M5" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="N5" s="33" t="s">
+      <c r="N5" s="32" t="s">
         <v>30</v>
       </c>
       <c r="O5" s="24" t="s">
@@ -18375,22 +18381,22 @@
       <c r="M6" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="33" t="s">
+      <c r="N6" s="32" t="s">
         <v>36</v>
       </c>
       <c r="O6" s="24" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:16380" ht="21" x14ac:dyDescent="0.4">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:16380" s="30" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A7" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
       <c r="E7" s="23" t="s">
         <v>11</v>
       </c>
@@ -18406,18 +18412,18 @@
       <c r="I7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="J7" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="31" t="s">
+      <c r="J7" s="28" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" s="34"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="35" t="s">
         <v>274</v>
       </c>
-      <c r="N7" s="9" t="s">
+      <c r="N7" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="O7" s="10" t="s">
+      <c r="O7" s="24" t="s">
         <v>26</v>
       </c>
     </row>
@@ -18428,7 +18434,7 @@
       <c r="B8" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="34"/>
+      <c r="C8" s="33"/>
       <c r="D8" s="20"/>
       <c r="E8" s="6" t="s">
         <v>11</v>
@@ -18450,7 +18456,7 @@
       </c>
       <c r="K8" s="11"/>
       <c r="L8" s="11"/>
-      <c r="M8" s="32" t="s">
+      <c r="M8" s="31" t="s">
         <v>43</v>
       </c>
       <c r="N8" s="9" t="s">
@@ -20365,15 +20371,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e3650b4f-99d5-4a38-9207-d1f63367a49d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="a44939b3-08bd-462e-9368-13442e4a2529" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="e3650b4f-99d5-4a38-9207-d1f63367a49d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -20590,21 +20593,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e3650b4f-99d5-4a38-9207-d1f63367a49d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="a44939b3-08bd-462e-9368-13442e4a2529" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="e3650b4f-99d5-4a38-9207-d1f63367a49d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F90BB4E-CB0E-4BCF-991B-A615C188294D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDAA5909-A9EB-412D-8D1A-52DA3BA11B01}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e3650b4f-99d5-4a38-9207-d1f63367a49d"/>
-    <ds:schemaRef ds:uri="a44939b3-08bd-462e-9368-13442e4a2529"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -20629,9 +20632,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDAA5909-A9EB-412D-8D1A-52DA3BA11B01}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F90BB4E-CB0E-4BCF-991B-A615C188294D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e3650b4f-99d5-4a38-9207-d1f63367a49d"/>
+    <ds:schemaRef ds:uri="a44939b3-08bd-462e-9368-13442e4a2529"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>